<commit_message>
feat: add raw data inventory
</commit_message>
<xml_diff>
--- a/data/metadata/data_inventory.xlsx
+++ b/data/metadata/data_inventory.xlsx
@@ -807,7 +807,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>저수지명 | 위치 | 유효저수량(천m3) | 2021-01-01 | 2021-01-02 | 2021-01-03 | 2021-01-04 | 2021-01-05 | 2021-01-06 | 2021-01-07 | 2021-01-08 | 2021-01-09 | 2021-01-10 | 2021-01-11 | 2021-01-12 | 2021-01-13 | 2021-01-14 | 2021-01-15 | 2021-01-16 | 2021-01-17 | 2021-01-18 | 2021-01-19 | 2021-01-20 | 2021-01-21 | 2021-01-22 | 2021-01-23 | 2021-01-24 | 2021-01-25 | 2021-01-26 | 2021-01-27</t>
+          <t>저수지명 | 위치 | 유효저수량(천m3) | 2021-01-01 | 2021-01-02 | 2021-01-03 | 2021-01-04 | 2021-01-05 | 2021-01-06 | 2021-01-07 | 2021-01-08 | 2021-01-09 | 2021-01-10 | 2021-01-11 | 2021-01-12 | 2021-01-13 | 2021-01-14 | 2021-01-15 | 2021-01-16 | 2021-01-17 | 2021-01-18 | 2021-01-19 | 2021-01-20 | 2021-01-21 | 2021-01-22 | 2021-01-23 | 2021-01-24 | 2021-01-25 | 2021-01-26 | 2021-01-27 | 2021-01-28 | 2021-01-29 | 2021-01-30 | 2021-01-31 | 2021-02-01 | 2021-02-02 | 2021-02-03 | 2021-02-04 | 2021-02-05 | 2021-02-06</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
@@ -855,7 +855,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>저수지명 | 위치 | 유효저수량(천m3) | 2023-01-01 | 2023-01-02 | 2023-01-03 | 2023-01-04 | 2023-01-05 | 2023-01-06 | 2023-01-07 | 2023-01-08 | 2023-01-09 | 2023-01-10 | 2023-01-11 | 2023-01-12 | 2023-01-13 | 2023-01-14 | 2023-01-15 | 2023-01-16 | 2023-01-17 | 2023-01-18 | 2023-01-19 | 2023-01-20 | 2023-01-21 | 2023-01-22 | 2023-01-23 | 2023-01-24 | 2023-01-25 | 2023-01-26 | 2023-01-27</t>
+          <t>저수지명 | 위치 | 유효저수량(천m3) | 2023-01-01 | 2023-01-02 | 2023-01-03 | 2023-01-04 | 2023-01-05 | 2023-01-06 | 2023-01-07 | 2023-01-08 | 2023-01-09 | 2023-01-10 | 2023-01-11 | 2023-01-12 | 2023-01-13 | 2023-01-14 | 2023-01-15 | 2023-01-16 | 2023-01-17 | 2023-01-18 | 2023-01-19 | 2023-01-20 | 2023-01-21 | 2023-01-22 | 2023-01-23 | 2023-01-24 | 2023-01-25 | 2023-01-26 | 2023-01-27 | 2023-01-28 | 2023-01-29 | 2023-01-30 | 2023-01-31 | 2023-02-01 | 2023-02-02 | 2023-02-03 | 2023-02-04 | 2023-02-05 | 2023-02-06</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
@@ -903,7 +903,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>저수지명 | 위치 | 유효저수량(천m3) | 2024-01-01 | 2024-01-02 | 2024-01-03 | 2024-01-04 | 2024-01-05 | 2024-01-06 | 2024-01-07 | 2024-01-08 | 2024-01-09 | 2024-01-10 | 2024-01-11 | 2024-01-12 | 2024-01-13 | 2024-01-14 | 2024-01-15 | 2024-01-16 | 2024-01-17 | 2024-01-18 | 2024-01-19 | 2024-01-20 | 2024-01-21 | 2024-01-22 | 2024-01-23 | 2024-01-24 | 2024-01-25 | 2024-01-26 | 2024-01-27</t>
+          <t>저수지명 | 위치 | 유효저수량(천m3) | 2024-01-01 | 2024-01-02 | 2024-01-03 | 2024-01-04 | 2024-01-05 | 2024-01-06 | 2024-01-07 | 2024-01-08 | 2024-01-09 | 2024-01-10 | 2024-01-11 | 2024-01-12 | 2024-01-13 | 2024-01-14 | 2024-01-15 | 2024-01-16 | 2024-01-17 | 2024-01-18 | 2024-01-19 | 2024-01-20 | 2024-01-21 | 2024-01-22 | 2024-01-23 | 2024-01-24 | 2024-01-25 | 2024-01-26 | 2024-01-27 | 2024-01-28 | 2024-01-29 | 2024-01-30 | 2024-01-31 | 2024-02-01 | 2024-02-02 | 2024-02-03 | 2024-02-04 | 2024-02-05 | 2024-02-06</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
@@ -951,7 +951,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>저수지명 | 위치 | 유효저수량(천m3) | 2022-01-01 | 2022-01-02 | 2022-01-03 | 2022-01-04 | 2022-01-05 | 2022-01-06 | 2022-01-07 | 2022-01-08 | 2022-01-09 | 2022-01-10 | 2022-01-11 | 2022-01-12 | 2022-01-13 | 2022-01-14 | 2022-01-15 | 2022-01-16 | 2022-01-17 | 2022-01-18 | 2022-01-19 | 2022-01-20 | 2022-01-21 | 2022-01-22 | 2022-01-23 | 2022-01-24 | 2022-01-25 | 2022-01-26 | 2022-01-27</t>
+          <t>저수지명 | 위치 | 유효저수량(천m3) | 2022-01-01 | 2022-01-02 | 2022-01-03 | 2022-01-04 | 2022-01-05 | 2022-01-06 | 2022-01-07 | 2022-01-08 | 2022-01-09 | 2022-01-10 | 2022-01-11 | 2022-01-12 | 2022-01-13 | 2022-01-14 | 2022-01-15 | 2022-01-16 | 2022-01-17 | 2022-01-18 | 2022-01-19 | 2022-01-20 | 2022-01-21 | 2022-01-22 | 2022-01-23 | 2022-01-24 | 2022-01-25 | 2022-01-26 | 2022-01-27 | 2022-01-28 | 2022-01-29 | 2022-01-30 | 2022-01-31 | 2022-02-01 | 2022-02-02 | 2022-02-03 | 2022-02-04 | 2022-02-05 | 2022-02-06</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
@@ -999,7 +999,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>저수지명 | 위치 | 유효저수량 | 2025-01-01 | 2025-01-02 | 2025-01-03 | 2025-01-04 | 2025-01-05 | 2025-01-06 | 2025-01-07 | 2025-01-08 | 2025-01-09 | 2025-01-10 | 2025-01-11 | 2025-01-12 | 2025-01-13 | 2025-01-14 | 2025-01-15 | 2025-01-16 | 2025-01-17 | 2025-01-18 | 2025-01-19 | 2025-01-20 | 2025-01-21 | 2025-01-22 | 2025-01-23 | 2025-01-24 | 2025-01-25 | 2025-01-26 | 2025-01-27</t>
+          <t>저수지명 | 위치 | 유효저수량 | 2025-01-01 | 2025-01-02 | 2025-01-03 | 2025-01-04 | 2025-01-05 | 2025-01-06 | 2025-01-07 | 2025-01-08 | 2025-01-09 | 2025-01-10 | 2025-01-11 | 2025-01-12 | 2025-01-13 | 2025-01-14 | 2025-01-15 | 2025-01-16 | 2025-01-17 | 2025-01-18 | 2025-01-19 | 2025-01-20 | 2025-01-21 | 2025-01-22 | 2025-01-23 | 2025-01-24 | 2025-01-25 | 2025-01-26 | 2025-01-27 | 2025-01-28 | 2025-01-29 | 2025-01-30 | 2025-01-31 | 2025-02-01 | 2025-02-02 | 2025-02-03 | 2025-02-04 | 2025-02-05 | 2025-02-06</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
@@ -1040,7 +1040,11 @@
           <t>2026-05-27 20:27:04</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>zip</t>
+        </is>
+      </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="n">
         <v>6</v>
@@ -1086,7 +1090,11 @@
           <t>2026-05-27 20:27:04</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>zip</t>
+        </is>
+      </c>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="n">
         <v>6</v>
@@ -1132,7 +1140,11 @@
           <t>2026-05-27 20:27:04</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>zip</t>
+        </is>
+      </c>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="n">
         <v>6</v>
@@ -1178,7 +1190,11 @@
           <t>2026-05-27 20:27:04</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>zip</t>
+        </is>
+      </c>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="n">
         <v>6</v>
@@ -1224,7 +1240,11 @@
           <t>2026-05-27 20:27:05</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>zip</t>
+        </is>
+      </c>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="n">
         <v>7</v>
@@ -1270,7 +1290,11 @@
           <t>2026-05-27 20:27:05</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>zip</t>
+        </is>
+      </c>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="n">
         <v>7</v>
@@ -1316,7 +1340,11 @@
           <t>2026-05-27 20:27:05</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>zip</t>
+        </is>
+      </c>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="n">
         <v>5</v>
@@ -1362,7 +1390,11 @@
           <t>2026-05-27 20:27:04</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>zip</t>
+        </is>
+      </c>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="n">
         <v>7</v>

</xml_diff>